<commit_message>
Linked &General activity creation completed
</commit_message>
<xml_diff>
--- a/SeleniumBDDFramework/src/test/resources/TestData/CRMActivityData.xlsx
+++ b/SeleniumBDDFramework/src/test/resources/TestData/CRMActivityData.xlsx
@@ -8,10 +8,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="General Activity" sheetId="1" r:id="rId1"/>
+    <sheet name="Linked Activity" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr/>
 </workbook>
@@ -74,6 +75,9 @@
     <t>I want to tag users for collaboration</t>
   </si>
   <si>
+    <t>Akash Mishra</t>
+  </si>
+  <si>
     <t>Physical Visit</t>
   </si>
   <si>
@@ -83,6 +87,9 @@
     <t>Vihaan Das</t>
   </si>
   <si>
+    <t>Keerthi Chowdary</t>
+  </si>
+  <si>
     <t>Virtual Visit</t>
   </si>
   <si>
@@ -92,6 +99,9 @@
     <t>Niharika Reddy</t>
   </si>
   <si>
+    <t>Surya Rana</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
@@ -99,13 +109,58 @@
   </si>
   <si>
     <t>Rahul Mishra</t>
+  </si>
+  <si>
+    <t>Rishi Kulkarni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead Name </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link to Stage </t>
+  </si>
+  <si>
+    <t>Little ville School</t>
+  </si>
+  <si>
+    <t>Demo</t>
+  </si>
+  <si>
+    <t>Created Linked Activity through Automation</t>
+  </si>
+  <si>
+    <t>Proposal</t>
+  </si>
+  <si>
+    <t>reports</t>
+  </si>
+  <si>
+    <t>Verbal Commitment</t>
+  </si>
+  <si>
+    <t>walkin</t>
+  </si>
+  <si>
+    <t>Deal Won</t>
+  </si>
+  <si>
+    <t>Zoom</t>
+  </si>
+  <si>
+    <t>Lead</t>
+  </si>
+  <si>
+    <t>Automated Linked activity</t>
+  </si>
+  <si>
+    <t>Audio</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,6 +213,13 @@
       <color theme="1"/>
       <name val="Poppins"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -224,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -241,6 +303,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -552,7 +619,7 @@
     <col min="5" max="5" width="15.29688" customWidth="1"/>
     <col min="6" max="6" width="16.29688" customWidth="1"/>
     <col min="7" max="7" width="42.09766" customWidth="1"/>
-    <col min="8" max="8" width="11.69922" customWidth="1"/>
+    <col min="8" max="8" width="26.5" customWidth="1"/>
     <col min="9" max="9" width="26.89844" customWidth="1"/>
   </cols>
   <sheetData>
@@ -663,13 +730,13 @@
         <v>17</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I4" s="11"/>
     </row>
     <row r="5" ht="17.4">
       <c r="A5" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>10</v>
@@ -678,7 +745,7 @@
         <v>11</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E5" s="9">
         <v>0.375</v>
@@ -694,7 +761,7 @@
     </row>
     <row r="6" ht="17.4">
       <c r="A6" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>10</v>
@@ -703,7 +770,7 @@
         <v>11</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E6" s="9">
         <v>0.41666666666666652</v>
@@ -715,7 +782,7 @@
         <v>14</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I6" s="11" t="s">
         <v>16</v>
@@ -723,7 +790,7 @@
     </row>
     <row r="7" ht="17.4">
       <c r="A7" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>10</v>
@@ -732,7 +799,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7" s="9">
         <v>0.54166666666666652</v>
@@ -744,13 +811,13 @@
         <v>17</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I7" s="11"/>
     </row>
     <row r="8" ht="17.4">
       <c r="A8" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>10</v>
@@ -759,7 +826,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E8" s="9">
         <v>0.375</v>
@@ -775,7 +842,7 @@
     </row>
     <row r="9" ht="17.4">
       <c r="A9" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>10</v>
@@ -784,7 +851,7 @@
         <v>11</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E9" s="9">
         <v>0.41666666666666652</v>
@@ -796,7 +863,7 @@
         <v>14</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I9" s="11" t="s">
         <v>16</v>
@@ -804,7 +871,7 @@
     </row>
     <row r="10" ht="17.4">
       <c r="A10" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>10</v>
@@ -813,7 +880,7 @@
         <v>11</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E10" s="9">
         <v>0.54166666666666652</v>
@@ -825,13 +892,13 @@
         <v>17</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I10" s="11"/>
     </row>
     <row r="11" ht="17.4">
       <c r="A11" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>10</v>
@@ -840,7 +907,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E11" s="9">
         <v>0.375</v>
@@ -856,7 +923,7 @@
     </row>
     <row r="12" ht="17.4">
       <c r="A12" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>10</v>
@@ -865,7 +932,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E12" s="9">
         <v>0.41666666666666652</v>
@@ -877,7 +944,7 @@
         <v>14</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>16</v>
@@ -885,7 +952,7 @@
     </row>
     <row r="13" ht="17.4">
       <c r="A13" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>10</v>
@@ -894,7 +961,7 @@
         <v>11</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E13" s="9">
         <v>0.54166666666666652</v>
@@ -906,9 +973,228 @@
         <v>17</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I13" s="11"/>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <cols>
+    <col min="1" max="1" width="16.29688" customWidth="1"/>
+    <col min="2" max="2" width="18.09766" customWidth="1"/>
+    <col min="3" max="3" width="12.79688" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="16.89844" customWidth="1"/>
+    <col min="6" max="6" width="11.5" customWidth="1"/>
+    <col min="7" max="7" width="14.89844" customWidth="1"/>
+    <col min="8" max="8" width="13.89844" customWidth="1"/>
+    <col min="9" max="9" width="29.29688" customWidth="1"/>
+    <col min="10" max="10" width="19.09766" customWidth="1"/>
+    <col min="11" max="11" width="22.69922" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.4">
+      <c r="A1" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" ht="17.4">
+      <c r="A2" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" s="18">
+        <v>46259</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0.375</v>
+      </c>
+      <c r="H2" s="9">
+        <v>0.41666666666666652</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+    </row>
+    <row r="3" ht="17.4">
+      <c r="A3" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="18">
+        <v>46260</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0.375</v>
+      </c>
+      <c r="H3" s="9">
+        <v>0.41666666666666652</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+    </row>
+    <row r="4" ht="17.4">
+      <c r="A4" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="18">
+        <v>46260</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0.54166666666666652</v>
+      </c>
+      <c r="H4" s="9">
+        <v>0.58333333333333326</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="11"/>
+    </row>
+    <row r="5" ht="27.6">
+      <c r="A5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="18">
+        <v>46261</v>
+      </c>
+      <c r="G5" s="9">
+        <v>0.41666666666666652</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0.45833333333333326</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" ht="17.4">
+      <c r="A6" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="18">
+        <v>46262</v>
+      </c>
+      <c r="G6" s="9">
+        <v>0.54166666666666652</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0.58333333333333326</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" s="11"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>